<commit_message>
Release container planner v2.3.0
</commit_message>
<xml_diff>
--- a/public/产品装柜规划导入模板.xlsx
+++ b/public/产品装柜规划导入模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品导入模板" sheetId="1" r:id="R7066cdb001574770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rc2c68220de45456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品导入模板" sheetId="1" r:id="Rc8ac7f9cbd25401f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R873e14bcd63f45f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -416,7 +416,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="9" t="str">
-        <x:v>家族</x:v>
+        <x:v>系列</x:v>
       </x:c>
       <x:c r="B1" s="10" t="str">
         <x:v>产品代码</x:v>
@@ -1168,10 +1168,10 @@
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="32" t="str">
-        <x:v>家族</x:v>
+        <x:v>系列</x:v>
       </x:c>
       <x:c r="B4" s="32" t="str">
-        <x:v>必填；产品家族编号或名称，例如 201、204/212</x:v>
+        <x:v>必填；产品系列编号或名称，例如 201、204/212</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">

</xml_diff>

<commit_message>
feat: harden mixed loading and report validation
</commit_message>
<xml_diff>
--- a/public/产品装柜规划导入模板.xlsx
+++ b/public/产品装柜规划导入模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品导入模板" sheetId="1" r:id="R07215c2d8ee94353"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R3c019644889b4825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品导入模板" sheetId="1" r:id="Rd181feedaa554765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R31d4c0f8bbc94637"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -557,7 +557,9 @@
       <x:c r="C2" s="15"/>
       <x:c r="D2" s="18"/>
       <x:c r="E2" s="18"/>
-      <x:c r="F2" s="15"/>
+      <x:c r="F2" s="15" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G2" s="21"/>
       <x:c r="H2" s="24"/>
     </x:row>
@@ -567,7 +569,9 @@
       <x:c r="C3" s="16"/>
       <x:c r="D3" s="19"/>
       <x:c r="E3" s="19"/>
-      <x:c r="F3" s="16"/>
+      <x:c r="F3" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G3" s="22"/>
       <x:c r="H3" s="25"/>
     </x:row>
@@ -577,7 +581,9 @@
       <x:c r="C4" s="16"/>
       <x:c r="D4" s="19"/>
       <x:c r="E4" s="19"/>
-      <x:c r="F4" s="16"/>
+      <x:c r="F4" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G4" s="22"/>
       <x:c r="H4" s="25"/>
     </x:row>
@@ -587,7 +593,9 @@
       <x:c r="C5" s="16"/>
       <x:c r="D5" s="19"/>
       <x:c r="E5" s="19"/>
-      <x:c r="F5" s="16"/>
+      <x:c r="F5" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G5" s="22"/>
       <x:c r="H5" s="25"/>
     </x:row>
@@ -597,7 +605,9 @@
       <x:c r="C6" s="16"/>
       <x:c r="D6" s="19"/>
       <x:c r="E6" s="19"/>
-      <x:c r="F6" s="16"/>
+      <x:c r="F6" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G6" s="22"/>
       <x:c r="H6" s="25"/>
     </x:row>
@@ -607,7 +617,9 @@
       <x:c r="C7" s="16"/>
       <x:c r="D7" s="19"/>
       <x:c r="E7" s="19"/>
-      <x:c r="F7" s="16"/>
+      <x:c r="F7" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G7" s="22"/>
       <x:c r="H7" s="25"/>
     </x:row>
@@ -617,7 +629,9 @@
       <x:c r="C8" s="16"/>
       <x:c r="D8" s="19"/>
       <x:c r="E8" s="19"/>
-      <x:c r="F8" s="16"/>
+      <x:c r="F8" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G8" s="22"/>
       <x:c r="H8" s="25"/>
     </x:row>
@@ -627,7 +641,9 @@
       <x:c r="C9" s="16"/>
       <x:c r="D9" s="19"/>
       <x:c r="E9" s="19"/>
-      <x:c r="F9" s="16"/>
+      <x:c r="F9" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G9" s="22"/>
       <x:c r="H9" s="25"/>
     </x:row>
@@ -637,7 +653,9 @@
       <x:c r="C10" s="16"/>
       <x:c r="D10" s="19"/>
       <x:c r="E10" s="19"/>
-      <x:c r="F10" s="16"/>
+      <x:c r="F10" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G10" s="22"/>
       <x:c r="H10" s="25"/>
     </x:row>
@@ -647,7 +665,9 @@
       <x:c r="C11" s="16"/>
       <x:c r="D11" s="19"/>
       <x:c r="E11" s="19"/>
-      <x:c r="F11" s="16"/>
+      <x:c r="F11" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G11" s="22"/>
       <x:c r="H11" s="25"/>
     </x:row>
@@ -657,7 +677,9 @@
       <x:c r="C12" s="16"/>
       <x:c r="D12" s="19"/>
       <x:c r="E12" s="19"/>
-      <x:c r="F12" s="16"/>
+      <x:c r="F12" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G12" s="22"/>
       <x:c r="H12" s="25"/>
     </x:row>
@@ -667,7 +689,9 @@
       <x:c r="C13" s="16"/>
       <x:c r="D13" s="19"/>
       <x:c r="E13" s="19"/>
-      <x:c r="F13" s="16"/>
+      <x:c r="F13" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G13" s="22"/>
       <x:c r="H13" s="25"/>
     </x:row>
@@ -677,7 +701,9 @@
       <x:c r="C14" s="16"/>
       <x:c r="D14" s="19"/>
       <x:c r="E14" s="19"/>
-      <x:c r="F14" s="16"/>
+      <x:c r="F14" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G14" s="22"/>
       <x:c r="H14" s="25"/>
     </x:row>
@@ -687,7 +713,9 @@
       <x:c r="C15" s="16"/>
       <x:c r="D15" s="19"/>
       <x:c r="E15" s="19"/>
-      <x:c r="F15" s="16"/>
+      <x:c r="F15" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G15" s="22"/>
       <x:c r="H15" s="25"/>
     </x:row>
@@ -697,7 +725,9 @@
       <x:c r="C16" s="16"/>
       <x:c r="D16" s="19"/>
       <x:c r="E16" s="19"/>
-      <x:c r="F16" s="16"/>
+      <x:c r="F16" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G16" s="22"/>
       <x:c r="H16" s="25"/>
     </x:row>
@@ -707,7 +737,9 @@
       <x:c r="C17" s="16"/>
       <x:c r="D17" s="19"/>
       <x:c r="E17" s="19"/>
-      <x:c r="F17" s="16"/>
+      <x:c r="F17" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G17" s="22"/>
       <x:c r="H17" s="25"/>
     </x:row>
@@ -717,7 +749,9 @@
       <x:c r="C18" s="16"/>
       <x:c r="D18" s="19"/>
       <x:c r="E18" s="19"/>
-      <x:c r="F18" s="16"/>
+      <x:c r="F18" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G18" s="22"/>
       <x:c r="H18" s="25"/>
     </x:row>
@@ -727,7 +761,9 @@
       <x:c r="C19" s="16"/>
       <x:c r="D19" s="19"/>
       <x:c r="E19" s="19"/>
-      <x:c r="F19" s="16"/>
+      <x:c r="F19" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G19" s="22"/>
       <x:c r="H19" s="25"/>
     </x:row>
@@ -737,7 +773,9 @@
       <x:c r="C20" s="16"/>
       <x:c r="D20" s="19"/>
       <x:c r="E20" s="19"/>
-      <x:c r="F20" s="16"/>
+      <x:c r="F20" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G20" s="22"/>
       <x:c r="H20" s="25"/>
     </x:row>
@@ -747,7 +785,9 @@
       <x:c r="C21" s="16"/>
       <x:c r="D21" s="19"/>
       <x:c r="E21" s="19"/>
-      <x:c r="F21" s="16"/>
+      <x:c r="F21" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G21" s="22"/>
       <x:c r="H21" s="25"/>
     </x:row>
@@ -757,7 +797,9 @@
       <x:c r="C22" s="16"/>
       <x:c r="D22" s="19"/>
       <x:c r="E22" s="19"/>
-      <x:c r="F22" s="16"/>
+      <x:c r="F22" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G22" s="22"/>
       <x:c r="H22" s="25"/>
     </x:row>
@@ -767,7 +809,9 @@
       <x:c r="C23" s="16"/>
       <x:c r="D23" s="19"/>
       <x:c r="E23" s="19"/>
-      <x:c r="F23" s="16"/>
+      <x:c r="F23" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G23" s="22"/>
       <x:c r="H23" s="25"/>
     </x:row>
@@ -777,7 +821,9 @@
       <x:c r="C24" s="16"/>
       <x:c r="D24" s="19"/>
       <x:c r="E24" s="19"/>
-      <x:c r="F24" s="16"/>
+      <x:c r="F24" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G24" s="22"/>
       <x:c r="H24" s="25"/>
     </x:row>
@@ -787,7 +833,9 @@
       <x:c r="C25" s="16"/>
       <x:c r="D25" s="19"/>
       <x:c r="E25" s="19"/>
-      <x:c r="F25" s="16"/>
+      <x:c r="F25" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G25" s="22"/>
       <x:c r="H25" s="25"/>
     </x:row>
@@ -797,7 +845,9 @@
       <x:c r="C26" s="16"/>
       <x:c r="D26" s="19"/>
       <x:c r="E26" s="19"/>
-      <x:c r="F26" s="16"/>
+      <x:c r="F26" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G26" s="22"/>
       <x:c r="H26" s="25"/>
     </x:row>
@@ -807,7 +857,9 @@
       <x:c r="C27" s="16"/>
       <x:c r="D27" s="19"/>
       <x:c r="E27" s="19"/>
-      <x:c r="F27" s="16"/>
+      <x:c r="F27" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G27" s="22"/>
       <x:c r="H27" s="25"/>
     </x:row>
@@ -817,7 +869,9 @@
       <x:c r="C28" s="16"/>
       <x:c r="D28" s="19"/>
       <x:c r="E28" s="19"/>
-      <x:c r="F28" s="16"/>
+      <x:c r="F28" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G28" s="22"/>
       <x:c r="H28" s="25"/>
     </x:row>
@@ -827,7 +881,9 @@
       <x:c r="C29" s="16"/>
       <x:c r="D29" s="19"/>
       <x:c r="E29" s="19"/>
-      <x:c r="F29" s="16"/>
+      <x:c r="F29" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G29" s="22"/>
       <x:c r="H29" s="25"/>
     </x:row>
@@ -837,7 +893,9 @@
       <x:c r="C30" s="16"/>
       <x:c r="D30" s="19"/>
       <x:c r="E30" s="19"/>
-      <x:c r="F30" s="16"/>
+      <x:c r="F30" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G30" s="22"/>
       <x:c r="H30" s="25"/>
     </x:row>
@@ -847,7 +905,9 @@
       <x:c r="C31" s="16"/>
       <x:c r="D31" s="19"/>
       <x:c r="E31" s="19"/>
-      <x:c r="F31" s="16"/>
+      <x:c r="F31" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G31" s="22"/>
       <x:c r="H31" s="25"/>
     </x:row>
@@ -857,7 +917,9 @@
       <x:c r="C32" s="16"/>
       <x:c r="D32" s="19"/>
       <x:c r="E32" s="19"/>
-      <x:c r="F32" s="16"/>
+      <x:c r="F32" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G32" s="22"/>
       <x:c r="H32" s="25"/>
     </x:row>
@@ -867,7 +929,9 @@
       <x:c r="C33" s="16"/>
       <x:c r="D33" s="19"/>
       <x:c r="E33" s="19"/>
-      <x:c r="F33" s="16"/>
+      <x:c r="F33" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G33" s="22"/>
       <x:c r="H33" s="25"/>
     </x:row>
@@ -877,7 +941,9 @@
       <x:c r="C34" s="16"/>
       <x:c r="D34" s="19"/>
       <x:c r="E34" s="19"/>
-      <x:c r="F34" s="16"/>
+      <x:c r="F34" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G34" s="22"/>
       <x:c r="H34" s="25"/>
     </x:row>
@@ -887,7 +953,9 @@
       <x:c r="C35" s="16"/>
       <x:c r="D35" s="19"/>
       <x:c r="E35" s="19"/>
-      <x:c r="F35" s="16"/>
+      <x:c r="F35" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G35" s="22"/>
       <x:c r="H35" s="25"/>
     </x:row>
@@ -897,7 +965,9 @@
       <x:c r="C36" s="16"/>
       <x:c r="D36" s="19"/>
       <x:c r="E36" s="19"/>
-      <x:c r="F36" s="16"/>
+      <x:c r="F36" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G36" s="22"/>
       <x:c r="H36" s="25"/>
     </x:row>
@@ -907,7 +977,9 @@
       <x:c r="C37" s="16"/>
       <x:c r="D37" s="19"/>
       <x:c r="E37" s="19"/>
-      <x:c r="F37" s="16"/>
+      <x:c r="F37" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G37" s="22"/>
       <x:c r="H37" s="25"/>
     </x:row>
@@ -917,7 +989,9 @@
       <x:c r="C38" s="16"/>
       <x:c r="D38" s="19"/>
       <x:c r="E38" s="19"/>
-      <x:c r="F38" s="16"/>
+      <x:c r="F38" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G38" s="22"/>
       <x:c r="H38" s="25"/>
     </x:row>
@@ -927,7 +1001,9 @@
       <x:c r="C39" s="16"/>
       <x:c r="D39" s="19"/>
       <x:c r="E39" s="19"/>
-      <x:c r="F39" s="16"/>
+      <x:c r="F39" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G39" s="22"/>
       <x:c r="H39" s="25"/>
     </x:row>
@@ -937,7 +1013,9 @@
       <x:c r="C40" s="16"/>
       <x:c r="D40" s="19"/>
       <x:c r="E40" s="19"/>
-      <x:c r="F40" s="16"/>
+      <x:c r="F40" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G40" s="22"/>
       <x:c r="H40" s="25"/>
     </x:row>
@@ -947,7 +1025,9 @@
       <x:c r="C41" s="16"/>
       <x:c r="D41" s="19"/>
       <x:c r="E41" s="19"/>
-      <x:c r="F41" s="16"/>
+      <x:c r="F41" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G41" s="22"/>
       <x:c r="H41" s="25"/>
     </x:row>
@@ -957,7 +1037,9 @@
       <x:c r="C42" s="16"/>
       <x:c r="D42" s="19"/>
       <x:c r="E42" s="19"/>
-      <x:c r="F42" s="16"/>
+      <x:c r="F42" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G42" s="22"/>
       <x:c r="H42" s="25"/>
     </x:row>
@@ -967,7 +1049,9 @@
       <x:c r="C43" s="16"/>
       <x:c r="D43" s="19"/>
       <x:c r="E43" s="19"/>
-      <x:c r="F43" s="16"/>
+      <x:c r="F43" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G43" s="22"/>
       <x:c r="H43" s="25"/>
     </x:row>
@@ -977,7 +1061,9 @@
       <x:c r="C44" s="16"/>
       <x:c r="D44" s="19"/>
       <x:c r="E44" s="19"/>
-      <x:c r="F44" s="16"/>
+      <x:c r="F44" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G44" s="22"/>
       <x:c r="H44" s="25"/>
     </x:row>
@@ -987,7 +1073,9 @@
       <x:c r="C45" s="16"/>
       <x:c r="D45" s="19"/>
       <x:c r="E45" s="19"/>
-      <x:c r="F45" s="16"/>
+      <x:c r="F45" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G45" s="22"/>
       <x:c r="H45" s="25"/>
     </x:row>
@@ -997,7 +1085,9 @@
       <x:c r="C46" s="16"/>
       <x:c r="D46" s="19"/>
       <x:c r="E46" s="19"/>
-      <x:c r="F46" s="16"/>
+      <x:c r="F46" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G46" s="22"/>
       <x:c r="H46" s="25"/>
     </x:row>
@@ -1007,7 +1097,9 @@
       <x:c r="C47" s="16"/>
       <x:c r="D47" s="19"/>
       <x:c r="E47" s="19"/>
-      <x:c r="F47" s="16"/>
+      <x:c r="F47" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G47" s="22"/>
       <x:c r="H47" s="25"/>
     </x:row>
@@ -1017,7 +1109,9 @@
       <x:c r="C48" s="16"/>
       <x:c r="D48" s="19"/>
       <x:c r="E48" s="19"/>
-      <x:c r="F48" s="16"/>
+      <x:c r="F48" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G48" s="22"/>
       <x:c r="H48" s="25"/>
     </x:row>
@@ -1027,7 +1121,9 @@
       <x:c r="C49" s="16"/>
       <x:c r="D49" s="19"/>
       <x:c r="E49" s="19"/>
-      <x:c r="F49" s="16"/>
+      <x:c r="F49" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G49" s="22"/>
       <x:c r="H49" s="25"/>
     </x:row>
@@ -1037,7 +1133,9 @@
       <x:c r="C50" s="16"/>
       <x:c r="D50" s="19"/>
       <x:c r="E50" s="19"/>
-      <x:c r="F50" s="16"/>
+      <x:c r="F50" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G50" s="22"/>
       <x:c r="H50" s="25"/>
     </x:row>
@@ -1047,7 +1145,9 @@
       <x:c r="C51" s="16"/>
       <x:c r="D51" s="19"/>
       <x:c r="E51" s="19"/>
-      <x:c r="F51" s="16"/>
+      <x:c r="F51" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G51" s="22"/>
       <x:c r="H51" s="25"/>
     </x:row>
@@ -1057,7 +1157,9 @@
       <x:c r="C52" s="16"/>
       <x:c r="D52" s="19"/>
       <x:c r="E52" s="19"/>
-      <x:c r="F52" s="16"/>
+      <x:c r="F52" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G52" s="22"/>
       <x:c r="H52" s="25"/>
     </x:row>
@@ -1067,7 +1169,9 @@
       <x:c r="C53" s="16"/>
       <x:c r="D53" s="19"/>
       <x:c r="E53" s="19"/>
-      <x:c r="F53" s="16"/>
+      <x:c r="F53" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G53" s="22"/>
       <x:c r="H53" s="25"/>
     </x:row>
@@ -1077,7 +1181,9 @@
       <x:c r="C54" s="16"/>
       <x:c r="D54" s="19"/>
       <x:c r="E54" s="19"/>
-      <x:c r="F54" s="16"/>
+      <x:c r="F54" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G54" s="22"/>
       <x:c r="H54" s="25"/>
     </x:row>
@@ -1087,7 +1193,9 @@
       <x:c r="C55" s="16"/>
       <x:c r="D55" s="19"/>
       <x:c r="E55" s="19"/>
-      <x:c r="F55" s="16"/>
+      <x:c r="F55" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G55" s="22"/>
       <x:c r="H55" s="25"/>
     </x:row>
@@ -1097,7 +1205,9 @@
       <x:c r="C56" s="16"/>
       <x:c r="D56" s="19"/>
       <x:c r="E56" s="19"/>
-      <x:c r="F56" s="16"/>
+      <x:c r="F56" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G56" s="22"/>
       <x:c r="H56" s="25"/>
     </x:row>
@@ -1107,7 +1217,9 @@
       <x:c r="C57" s="16"/>
       <x:c r="D57" s="19"/>
       <x:c r="E57" s="19"/>
-      <x:c r="F57" s="16"/>
+      <x:c r="F57" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G57" s="22"/>
       <x:c r="H57" s="25"/>
     </x:row>
@@ -1117,7 +1229,9 @@
       <x:c r="C58" s="16"/>
       <x:c r="D58" s="19"/>
       <x:c r="E58" s="19"/>
-      <x:c r="F58" s="16"/>
+      <x:c r="F58" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G58" s="22"/>
       <x:c r="H58" s="25"/>
     </x:row>
@@ -1127,7 +1241,9 @@
       <x:c r="C59" s="16"/>
       <x:c r="D59" s="19"/>
       <x:c r="E59" s="19"/>
-      <x:c r="F59" s="16"/>
+      <x:c r="F59" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G59" s="22"/>
       <x:c r="H59" s="25"/>
     </x:row>
@@ -1137,7 +1253,9 @@
       <x:c r="C60" s="16"/>
       <x:c r="D60" s="19"/>
       <x:c r="E60" s="19"/>
-      <x:c r="F60" s="16"/>
+      <x:c r="F60" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G60" s="22"/>
       <x:c r="H60" s="25"/>
     </x:row>
@@ -1147,7 +1265,9 @@
       <x:c r="C61" s="16"/>
       <x:c r="D61" s="19"/>
       <x:c r="E61" s="19"/>
-      <x:c r="F61" s="16"/>
+      <x:c r="F61" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G61" s="22"/>
       <x:c r="H61" s="25"/>
     </x:row>
@@ -1157,7 +1277,9 @@
       <x:c r="C62" s="16"/>
       <x:c r="D62" s="19"/>
       <x:c r="E62" s="19"/>
-      <x:c r="F62" s="16"/>
+      <x:c r="F62" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G62" s="22"/>
       <x:c r="H62" s="25"/>
     </x:row>
@@ -1167,7 +1289,9 @@
       <x:c r="C63" s="16"/>
       <x:c r="D63" s="19"/>
       <x:c r="E63" s="19"/>
-      <x:c r="F63" s="16"/>
+      <x:c r="F63" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G63" s="22"/>
       <x:c r="H63" s="25"/>
     </x:row>
@@ -1177,7 +1301,9 @@
       <x:c r="C64" s="16"/>
       <x:c r="D64" s="19"/>
       <x:c r="E64" s="19"/>
-      <x:c r="F64" s="16"/>
+      <x:c r="F64" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G64" s="22"/>
       <x:c r="H64" s="25"/>
     </x:row>
@@ -1187,7 +1313,9 @@
       <x:c r="C65" s="16"/>
       <x:c r="D65" s="19"/>
       <x:c r="E65" s="19"/>
-      <x:c r="F65" s="16"/>
+      <x:c r="F65" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G65" s="22"/>
       <x:c r="H65" s="25"/>
     </x:row>
@@ -1197,7 +1325,9 @@
       <x:c r="C66" s="16"/>
       <x:c r="D66" s="19"/>
       <x:c r="E66" s="19"/>
-      <x:c r="F66" s="16"/>
+      <x:c r="F66" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G66" s="22"/>
       <x:c r="H66" s="25"/>
     </x:row>
@@ -1207,7 +1337,9 @@
       <x:c r="C67" s="16"/>
       <x:c r="D67" s="19"/>
       <x:c r="E67" s="19"/>
-      <x:c r="F67" s="16"/>
+      <x:c r="F67" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G67" s="22"/>
       <x:c r="H67" s="25"/>
     </x:row>
@@ -1217,7 +1349,9 @@
       <x:c r="C68" s="16"/>
       <x:c r="D68" s="19"/>
       <x:c r="E68" s="19"/>
-      <x:c r="F68" s="16"/>
+      <x:c r="F68" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G68" s="22"/>
       <x:c r="H68" s="25"/>
     </x:row>
@@ -1227,7 +1361,9 @@
       <x:c r="C69" s="16"/>
       <x:c r="D69" s="19"/>
       <x:c r="E69" s="19"/>
-      <x:c r="F69" s="16"/>
+      <x:c r="F69" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G69" s="22"/>
       <x:c r="H69" s="25"/>
     </x:row>
@@ -1237,7 +1373,9 @@
       <x:c r="C70" s="16"/>
       <x:c r="D70" s="19"/>
       <x:c r="E70" s="19"/>
-      <x:c r="F70" s="16"/>
+      <x:c r="F70" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G70" s="22"/>
       <x:c r="H70" s="25"/>
     </x:row>
@@ -1247,7 +1385,9 @@
       <x:c r="C71" s="16"/>
       <x:c r="D71" s="19"/>
       <x:c r="E71" s="19"/>
-      <x:c r="F71" s="16"/>
+      <x:c r="F71" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G71" s="22"/>
       <x:c r="H71" s="25"/>
     </x:row>
@@ -1257,7 +1397,9 @@
       <x:c r="C72" s="16"/>
       <x:c r="D72" s="19"/>
       <x:c r="E72" s="19"/>
-      <x:c r="F72" s="16"/>
+      <x:c r="F72" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G72" s="22"/>
       <x:c r="H72" s="25"/>
     </x:row>
@@ -1267,7 +1409,9 @@
       <x:c r="C73" s="16"/>
       <x:c r="D73" s="19"/>
       <x:c r="E73" s="19"/>
-      <x:c r="F73" s="16"/>
+      <x:c r="F73" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G73" s="22"/>
       <x:c r="H73" s="25"/>
     </x:row>
@@ -1277,7 +1421,9 @@
       <x:c r="C74" s="16"/>
       <x:c r="D74" s="19"/>
       <x:c r="E74" s="19"/>
-      <x:c r="F74" s="16"/>
+      <x:c r="F74" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G74" s="22"/>
       <x:c r="H74" s="25"/>
     </x:row>
@@ -1287,7 +1433,9 @@
       <x:c r="C75" s="16"/>
       <x:c r="D75" s="19"/>
       <x:c r="E75" s="19"/>
-      <x:c r="F75" s="16"/>
+      <x:c r="F75" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G75" s="22"/>
       <x:c r="H75" s="25"/>
     </x:row>
@@ -1297,7 +1445,9 @@
       <x:c r="C76" s="16"/>
       <x:c r="D76" s="19"/>
       <x:c r="E76" s="19"/>
-      <x:c r="F76" s="16"/>
+      <x:c r="F76" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G76" s="22"/>
       <x:c r="H76" s="25"/>
     </x:row>
@@ -1307,7 +1457,9 @@
       <x:c r="C77" s="16"/>
       <x:c r="D77" s="19"/>
       <x:c r="E77" s="19"/>
-      <x:c r="F77" s="16"/>
+      <x:c r="F77" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G77" s="22"/>
       <x:c r="H77" s="25"/>
     </x:row>
@@ -1317,7 +1469,9 @@
       <x:c r="C78" s="16"/>
       <x:c r="D78" s="19"/>
       <x:c r="E78" s="19"/>
-      <x:c r="F78" s="16"/>
+      <x:c r="F78" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G78" s="22"/>
       <x:c r="H78" s="25"/>
     </x:row>
@@ -1327,7 +1481,9 @@
       <x:c r="C79" s="16"/>
       <x:c r="D79" s="19"/>
       <x:c r="E79" s="19"/>
-      <x:c r="F79" s="16"/>
+      <x:c r="F79" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G79" s="22"/>
       <x:c r="H79" s="25"/>
     </x:row>
@@ -1337,7 +1493,9 @@
       <x:c r="C80" s="16"/>
       <x:c r="D80" s="19"/>
       <x:c r="E80" s="19"/>
-      <x:c r="F80" s="16"/>
+      <x:c r="F80" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G80" s="22"/>
       <x:c r="H80" s="25"/>
     </x:row>
@@ -1347,7 +1505,9 @@
       <x:c r="C81" s="16"/>
       <x:c r="D81" s="19"/>
       <x:c r="E81" s="19"/>
-      <x:c r="F81" s="16"/>
+      <x:c r="F81" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G81" s="22"/>
       <x:c r="H81" s="25"/>
     </x:row>
@@ -1357,7 +1517,9 @@
       <x:c r="C82" s="16"/>
       <x:c r="D82" s="19"/>
       <x:c r="E82" s="19"/>
-      <x:c r="F82" s="16"/>
+      <x:c r="F82" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G82" s="22"/>
       <x:c r="H82" s="25"/>
     </x:row>
@@ -1367,7 +1529,9 @@
       <x:c r="C83" s="16"/>
       <x:c r="D83" s="19"/>
       <x:c r="E83" s="19"/>
-      <x:c r="F83" s="16"/>
+      <x:c r="F83" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G83" s="22"/>
       <x:c r="H83" s="25"/>
     </x:row>
@@ -1377,7 +1541,9 @@
       <x:c r="C84" s="16"/>
       <x:c r="D84" s="19"/>
       <x:c r="E84" s="19"/>
-      <x:c r="F84" s="16"/>
+      <x:c r="F84" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G84" s="22"/>
       <x:c r="H84" s="25"/>
     </x:row>
@@ -1387,7 +1553,9 @@
       <x:c r="C85" s="16"/>
       <x:c r="D85" s="19"/>
       <x:c r="E85" s="19"/>
-      <x:c r="F85" s="16"/>
+      <x:c r="F85" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G85" s="22"/>
       <x:c r="H85" s="25"/>
     </x:row>
@@ -1397,7 +1565,9 @@
       <x:c r="C86" s="16"/>
       <x:c r="D86" s="19"/>
       <x:c r="E86" s="19"/>
-      <x:c r="F86" s="16"/>
+      <x:c r="F86" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G86" s="22"/>
       <x:c r="H86" s="25"/>
     </x:row>
@@ -1407,7 +1577,9 @@
       <x:c r="C87" s="16"/>
       <x:c r="D87" s="19"/>
       <x:c r="E87" s="19"/>
-      <x:c r="F87" s="16"/>
+      <x:c r="F87" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G87" s="22"/>
       <x:c r="H87" s="25"/>
     </x:row>
@@ -1417,7 +1589,9 @@
       <x:c r="C88" s="16"/>
       <x:c r="D88" s="19"/>
       <x:c r="E88" s="19"/>
-      <x:c r="F88" s="16"/>
+      <x:c r="F88" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G88" s="22"/>
       <x:c r="H88" s="25"/>
     </x:row>
@@ -1427,7 +1601,9 @@
       <x:c r="C89" s="16"/>
       <x:c r="D89" s="19"/>
       <x:c r="E89" s="19"/>
-      <x:c r="F89" s="16"/>
+      <x:c r="F89" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G89" s="22"/>
       <x:c r="H89" s="25"/>
     </x:row>
@@ -1437,7 +1613,9 @@
       <x:c r="C90" s="16"/>
       <x:c r="D90" s="19"/>
       <x:c r="E90" s="19"/>
-      <x:c r="F90" s="16"/>
+      <x:c r="F90" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G90" s="22"/>
       <x:c r="H90" s="25"/>
     </x:row>
@@ -1447,7 +1625,9 @@
       <x:c r="C91" s="16"/>
       <x:c r="D91" s="19"/>
       <x:c r="E91" s="19"/>
-      <x:c r="F91" s="16"/>
+      <x:c r="F91" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G91" s="22"/>
       <x:c r="H91" s="25"/>
     </x:row>
@@ -1457,7 +1637,9 @@
       <x:c r="C92" s="16"/>
       <x:c r="D92" s="19"/>
       <x:c r="E92" s="19"/>
-      <x:c r="F92" s="16"/>
+      <x:c r="F92" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G92" s="22"/>
       <x:c r="H92" s="25"/>
     </x:row>
@@ -1467,7 +1649,9 @@
       <x:c r="C93" s="16"/>
       <x:c r="D93" s="19"/>
       <x:c r="E93" s="19"/>
-      <x:c r="F93" s="16"/>
+      <x:c r="F93" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G93" s="22"/>
       <x:c r="H93" s="25"/>
     </x:row>
@@ -1477,7 +1661,9 @@
       <x:c r="C94" s="16"/>
       <x:c r="D94" s="19"/>
       <x:c r="E94" s="19"/>
-      <x:c r="F94" s="16"/>
+      <x:c r="F94" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G94" s="22"/>
       <x:c r="H94" s="25"/>
     </x:row>
@@ -1487,7 +1673,9 @@
       <x:c r="C95" s="16"/>
       <x:c r="D95" s="19"/>
       <x:c r="E95" s="19"/>
-      <x:c r="F95" s="16"/>
+      <x:c r="F95" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G95" s="22"/>
       <x:c r="H95" s="25"/>
     </x:row>
@@ -1497,7 +1685,9 @@
       <x:c r="C96" s="16"/>
       <x:c r="D96" s="19"/>
       <x:c r="E96" s="19"/>
-      <x:c r="F96" s="16"/>
+      <x:c r="F96" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G96" s="22"/>
       <x:c r="H96" s="25"/>
     </x:row>
@@ -1507,7 +1697,9 @@
       <x:c r="C97" s="16"/>
       <x:c r="D97" s="19"/>
       <x:c r="E97" s="19"/>
-      <x:c r="F97" s="16"/>
+      <x:c r="F97" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G97" s="22"/>
       <x:c r="H97" s="25"/>
     </x:row>
@@ -1517,7 +1709,9 @@
       <x:c r="C98" s="16"/>
       <x:c r="D98" s="19"/>
       <x:c r="E98" s="19"/>
-      <x:c r="F98" s="16"/>
+      <x:c r="F98" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G98" s="22"/>
       <x:c r="H98" s="25"/>
     </x:row>
@@ -1527,7 +1721,9 @@
       <x:c r="C99" s="16"/>
       <x:c r="D99" s="19"/>
       <x:c r="E99" s="19"/>
-      <x:c r="F99" s="16"/>
+      <x:c r="F99" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G99" s="22"/>
       <x:c r="H99" s="25"/>
     </x:row>
@@ -1537,7 +1733,9 @@
       <x:c r="C100" s="16"/>
       <x:c r="D100" s="19"/>
       <x:c r="E100" s="19"/>
-      <x:c r="F100" s="16"/>
+      <x:c r="F100" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G100" s="22"/>
       <x:c r="H100" s="25"/>
     </x:row>
@@ -1547,7 +1745,9 @@
       <x:c r="C101" s="16"/>
       <x:c r="D101" s="19"/>
       <x:c r="E101" s="19"/>
-      <x:c r="F101" s="16"/>
+      <x:c r="F101" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G101" s="22"/>
       <x:c r="H101" s="25"/>
     </x:row>
@@ -1557,7 +1757,9 @@
       <x:c r="C102" s="16"/>
       <x:c r="D102" s="19"/>
       <x:c r="E102" s="19"/>
-      <x:c r="F102" s="16"/>
+      <x:c r="F102" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G102" s="22"/>
       <x:c r="H102" s="25"/>
     </x:row>
@@ -1567,7 +1769,9 @@
       <x:c r="C103" s="16"/>
       <x:c r="D103" s="19"/>
       <x:c r="E103" s="19"/>
-      <x:c r="F103" s="16"/>
+      <x:c r="F103" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G103" s="22"/>
       <x:c r="H103" s="25"/>
     </x:row>
@@ -1577,7 +1781,9 @@
       <x:c r="C104" s="16"/>
       <x:c r="D104" s="19"/>
       <x:c r="E104" s="19"/>
-      <x:c r="F104" s="16"/>
+      <x:c r="F104" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G104" s="22"/>
       <x:c r="H104" s="25"/>
     </x:row>
@@ -1587,7 +1793,9 @@
       <x:c r="C105" s="16"/>
       <x:c r="D105" s="19"/>
       <x:c r="E105" s="19"/>
-      <x:c r="F105" s="16"/>
+      <x:c r="F105" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G105" s="22"/>
       <x:c r="H105" s="25"/>
     </x:row>
@@ -1597,7 +1805,9 @@
       <x:c r="C106" s="16"/>
       <x:c r="D106" s="19"/>
       <x:c r="E106" s="19"/>
-      <x:c r="F106" s="16"/>
+      <x:c r="F106" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G106" s="22"/>
       <x:c r="H106" s="25"/>
     </x:row>
@@ -1607,7 +1817,9 @@
       <x:c r="C107" s="16"/>
       <x:c r="D107" s="19"/>
       <x:c r="E107" s="19"/>
-      <x:c r="F107" s="16"/>
+      <x:c r="F107" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G107" s="22"/>
       <x:c r="H107" s="25"/>
     </x:row>
@@ -1617,7 +1829,9 @@
       <x:c r="C108" s="16"/>
       <x:c r="D108" s="19"/>
       <x:c r="E108" s="19"/>
-      <x:c r="F108" s="16"/>
+      <x:c r="F108" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G108" s="22"/>
       <x:c r="H108" s="25"/>
     </x:row>
@@ -1627,7 +1841,9 @@
       <x:c r="C109" s="16"/>
       <x:c r="D109" s="19"/>
       <x:c r="E109" s="19"/>
-      <x:c r="F109" s="16"/>
+      <x:c r="F109" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G109" s="22"/>
       <x:c r="H109" s="25"/>
     </x:row>
@@ -1637,7 +1853,9 @@
       <x:c r="C110" s="16"/>
       <x:c r="D110" s="19"/>
       <x:c r="E110" s="19"/>
-      <x:c r="F110" s="16"/>
+      <x:c r="F110" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G110" s="22"/>
       <x:c r="H110" s="25"/>
     </x:row>
@@ -1647,7 +1865,9 @@
       <x:c r="C111" s="16"/>
       <x:c r="D111" s="19"/>
       <x:c r="E111" s="19"/>
-      <x:c r="F111" s="16"/>
+      <x:c r="F111" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G111" s="22"/>
       <x:c r="H111" s="25"/>
     </x:row>
@@ -1657,7 +1877,9 @@
       <x:c r="C112" s="16"/>
       <x:c r="D112" s="19"/>
       <x:c r="E112" s="19"/>
-      <x:c r="F112" s="16"/>
+      <x:c r="F112" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G112" s="22"/>
       <x:c r="H112" s="25"/>
     </x:row>
@@ -1667,7 +1889,9 @@
       <x:c r="C113" s="16"/>
       <x:c r="D113" s="19"/>
       <x:c r="E113" s="19"/>
-      <x:c r="F113" s="16"/>
+      <x:c r="F113" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G113" s="22"/>
       <x:c r="H113" s="25"/>
     </x:row>
@@ -1677,7 +1901,9 @@
       <x:c r="C114" s="16"/>
       <x:c r="D114" s="19"/>
       <x:c r="E114" s="19"/>
-      <x:c r="F114" s="16"/>
+      <x:c r="F114" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G114" s="22"/>
       <x:c r="H114" s="25"/>
     </x:row>
@@ -1687,7 +1913,9 @@
       <x:c r="C115" s="16"/>
       <x:c r="D115" s="19"/>
       <x:c r="E115" s="19"/>
-      <x:c r="F115" s="16"/>
+      <x:c r="F115" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G115" s="22"/>
       <x:c r="H115" s="25"/>
     </x:row>
@@ -1697,7 +1925,9 @@
       <x:c r="C116" s="16"/>
       <x:c r="D116" s="19"/>
       <x:c r="E116" s="19"/>
-      <x:c r="F116" s="16"/>
+      <x:c r="F116" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G116" s="22"/>
       <x:c r="H116" s="25"/>
     </x:row>
@@ -1707,7 +1937,9 @@
       <x:c r="C117" s="16"/>
       <x:c r="D117" s="19"/>
       <x:c r="E117" s="19"/>
-      <x:c r="F117" s="16"/>
+      <x:c r="F117" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G117" s="22"/>
       <x:c r="H117" s="25"/>
     </x:row>
@@ -1717,7 +1949,9 @@
       <x:c r="C118" s="16"/>
       <x:c r="D118" s="19"/>
       <x:c r="E118" s="19"/>
-      <x:c r="F118" s="16"/>
+      <x:c r="F118" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G118" s="22"/>
       <x:c r="H118" s="25"/>
     </x:row>
@@ -1727,7 +1961,9 @@
       <x:c r="C119" s="16"/>
       <x:c r="D119" s="19"/>
       <x:c r="E119" s="19"/>
-      <x:c r="F119" s="16"/>
+      <x:c r="F119" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G119" s="22"/>
       <x:c r="H119" s="25"/>
     </x:row>
@@ -1737,7 +1973,9 @@
       <x:c r="C120" s="16"/>
       <x:c r="D120" s="19"/>
       <x:c r="E120" s="19"/>
-      <x:c r="F120" s="16"/>
+      <x:c r="F120" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G120" s="22"/>
       <x:c r="H120" s="25"/>
     </x:row>
@@ -1747,7 +1985,9 @@
       <x:c r="C121" s="16"/>
       <x:c r="D121" s="19"/>
       <x:c r="E121" s="19"/>
-      <x:c r="F121" s="16"/>
+      <x:c r="F121" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G121" s="22"/>
       <x:c r="H121" s="25"/>
     </x:row>
@@ -1757,7 +1997,9 @@
       <x:c r="C122" s="16"/>
       <x:c r="D122" s="19"/>
       <x:c r="E122" s="19"/>
-      <x:c r="F122" s="16"/>
+      <x:c r="F122" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G122" s="22"/>
       <x:c r="H122" s="25"/>
     </x:row>
@@ -1767,7 +2009,9 @@
       <x:c r="C123" s="16"/>
       <x:c r="D123" s="19"/>
       <x:c r="E123" s="19"/>
-      <x:c r="F123" s="16"/>
+      <x:c r="F123" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G123" s="22"/>
       <x:c r="H123" s="25"/>
     </x:row>
@@ -1777,7 +2021,9 @@
       <x:c r="C124" s="16"/>
       <x:c r="D124" s="19"/>
       <x:c r="E124" s="19"/>
-      <x:c r="F124" s="16"/>
+      <x:c r="F124" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G124" s="22"/>
       <x:c r="H124" s="25"/>
     </x:row>
@@ -1787,7 +2033,9 @@
       <x:c r="C125" s="16"/>
       <x:c r="D125" s="19"/>
       <x:c r="E125" s="19"/>
-      <x:c r="F125" s="16"/>
+      <x:c r="F125" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G125" s="22"/>
       <x:c r="H125" s="25"/>
     </x:row>
@@ -1797,7 +2045,9 @@
       <x:c r="C126" s="16"/>
       <x:c r="D126" s="19"/>
       <x:c r="E126" s="19"/>
-      <x:c r="F126" s="16"/>
+      <x:c r="F126" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G126" s="22"/>
       <x:c r="H126" s="25"/>
     </x:row>
@@ -1807,7 +2057,9 @@
       <x:c r="C127" s="16"/>
       <x:c r="D127" s="19"/>
       <x:c r="E127" s="19"/>
-      <x:c r="F127" s="16"/>
+      <x:c r="F127" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G127" s="22"/>
       <x:c r="H127" s="25"/>
     </x:row>
@@ -1817,7 +2069,9 @@
       <x:c r="C128" s="16"/>
       <x:c r="D128" s="19"/>
       <x:c r="E128" s="19"/>
-      <x:c r="F128" s="16"/>
+      <x:c r="F128" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G128" s="22"/>
       <x:c r="H128" s="25"/>
     </x:row>
@@ -1827,7 +2081,9 @@
       <x:c r="C129" s="16"/>
       <x:c r="D129" s="19"/>
       <x:c r="E129" s="19"/>
-      <x:c r="F129" s="16"/>
+      <x:c r="F129" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G129" s="22"/>
       <x:c r="H129" s="25"/>
     </x:row>
@@ -1837,7 +2093,9 @@
       <x:c r="C130" s="16"/>
       <x:c r="D130" s="19"/>
       <x:c r="E130" s="19"/>
-      <x:c r="F130" s="16"/>
+      <x:c r="F130" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G130" s="22"/>
       <x:c r="H130" s="25"/>
     </x:row>
@@ -1847,7 +2105,9 @@
       <x:c r="C131" s="16"/>
       <x:c r="D131" s="19"/>
       <x:c r="E131" s="19"/>
-      <x:c r="F131" s="16"/>
+      <x:c r="F131" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G131" s="22"/>
       <x:c r="H131" s="25"/>
     </x:row>
@@ -1857,7 +2117,9 @@
       <x:c r="C132" s="16"/>
       <x:c r="D132" s="19"/>
       <x:c r="E132" s="19"/>
-      <x:c r="F132" s="16"/>
+      <x:c r="F132" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G132" s="22"/>
       <x:c r="H132" s="25"/>
     </x:row>
@@ -1867,7 +2129,9 @@
       <x:c r="C133" s="16"/>
       <x:c r="D133" s="19"/>
       <x:c r="E133" s="19"/>
-      <x:c r="F133" s="16"/>
+      <x:c r="F133" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G133" s="22"/>
       <x:c r="H133" s="25"/>
     </x:row>
@@ -1877,7 +2141,9 @@
       <x:c r="C134" s="16"/>
       <x:c r="D134" s="19"/>
       <x:c r="E134" s="19"/>
-      <x:c r="F134" s="16"/>
+      <x:c r="F134" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G134" s="22"/>
       <x:c r="H134" s="25"/>
     </x:row>
@@ -1887,7 +2153,9 @@
       <x:c r="C135" s="16"/>
       <x:c r="D135" s="19"/>
       <x:c r="E135" s="19"/>
-      <x:c r="F135" s="16"/>
+      <x:c r="F135" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G135" s="22"/>
       <x:c r="H135" s="25"/>
     </x:row>
@@ -1897,7 +2165,9 @@
       <x:c r="C136" s="16"/>
       <x:c r="D136" s="19"/>
       <x:c r="E136" s="19"/>
-      <x:c r="F136" s="16"/>
+      <x:c r="F136" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G136" s="22"/>
       <x:c r="H136" s="25"/>
     </x:row>
@@ -1907,7 +2177,9 @@
       <x:c r="C137" s="16"/>
       <x:c r="D137" s="19"/>
       <x:c r="E137" s="19"/>
-      <x:c r="F137" s="16"/>
+      <x:c r="F137" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G137" s="22"/>
       <x:c r="H137" s="25"/>
     </x:row>
@@ -1917,7 +2189,9 @@
       <x:c r="C138" s="16"/>
       <x:c r="D138" s="19"/>
       <x:c r="E138" s="19"/>
-      <x:c r="F138" s="16"/>
+      <x:c r="F138" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G138" s="22"/>
       <x:c r="H138" s="25"/>
     </x:row>
@@ -1927,7 +2201,9 @@
       <x:c r="C139" s="16"/>
       <x:c r="D139" s="19"/>
       <x:c r="E139" s="19"/>
-      <x:c r="F139" s="16"/>
+      <x:c r="F139" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G139" s="22"/>
       <x:c r="H139" s="25"/>
     </x:row>
@@ -1937,7 +2213,9 @@
       <x:c r="C140" s="16"/>
       <x:c r="D140" s="19"/>
       <x:c r="E140" s="19"/>
-      <x:c r="F140" s="16"/>
+      <x:c r="F140" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G140" s="22"/>
       <x:c r="H140" s="25"/>
     </x:row>
@@ -1947,7 +2225,9 @@
       <x:c r="C141" s="16"/>
       <x:c r="D141" s="19"/>
       <x:c r="E141" s="19"/>
-      <x:c r="F141" s="16"/>
+      <x:c r="F141" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G141" s="22"/>
       <x:c r="H141" s="25"/>
     </x:row>
@@ -1957,7 +2237,9 @@
       <x:c r="C142" s="16"/>
       <x:c r="D142" s="19"/>
       <x:c r="E142" s="19"/>
-      <x:c r="F142" s="16"/>
+      <x:c r="F142" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G142" s="22"/>
       <x:c r="H142" s="25"/>
     </x:row>
@@ -1967,7 +2249,9 @@
       <x:c r="C143" s="16"/>
       <x:c r="D143" s="19"/>
       <x:c r="E143" s="19"/>
-      <x:c r="F143" s="16"/>
+      <x:c r="F143" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G143" s="22"/>
       <x:c r="H143" s="25"/>
     </x:row>
@@ -1977,7 +2261,9 @@
       <x:c r="C144" s="16"/>
       <x:c r="D144" s="19"/>
       <x:c r="E144" s="19"/>
-      <x:c r="F144" s="16"/>
+      <x:c r="F144" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G144" s="22"/>
       <x:c r="H144" s="25"/>
     </x:row>
@@ -1987,7 +2273,9 @@
       <x:c r="C145" s="16"/>
       <x:c r="D145" s="19"/>
       <x:c r="E145" s="19"/>
-      <x:c r="F145" s="16"/>
+      <x:c r="F145" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G145" s="22"/>
       <x:c r="H145" s="25"/>
     </x:row>
@@ -1997,7 +2285,9 @@
       <x:c r="C146" s="16"/>
       <x:c r="D146" s="19"/>
       <x:c r="E146" s="19"/>
-      <x:c r="F146" s="16"/>
+      <x:c r="F146" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G146" s="22"/>
       <x:c r="H146" s="25"/>
     </x:row>
@@ -2007,7 +2297,9 @@
       <x:c r="C147" s="16"/>
       <x:c r="D147" s="19"/>
       <x:c r="E147" s="19"/>
-      <x:c r="F147" s="16"/>
+      <x:c r="F147" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G147" s="22"/>
       <x:c r="H147" s="25"/>
     </x:row>
@@ -2017,7 +2309,9 @@
       <x:c r="C148" s="16"/>
       <x:c r="D148" s="19"/>
       <x:c r="E148" s="19"/>
-      <x:c r="F148" s="16"/>
+      <x:c r="F148" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G148" s="22"/>
       <x:c r="H148" s="25"/>
     </x:row>
@@ -2027,7 +2321,9 @@
       <x:c r="C149" s="16"/>
       <x:c r="D149" s="19"/>
       <x:c r="E149" s="19"/>
-      <x:c r="F149" s="16"/>
+      <x:c r="F149" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G149" s="22"/>
       <x:c r="H149" s="25"/>
     </x:row>
@@ -2037,7 +2333,9 @@
       <x:c r="C150" s="16"/>
       <x:c r="D150" s="19"/>
       <x:c r="E150" s="19"/>
-      <x:c r="F150" s="16"/>
+      <x:c r="F150" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G150" s="22"/>
       <x:c r="H150" s="25"/>
     </x:row>
@@ -2047,7 +2345,9 @@
       <x:c r="C151" s="16"/>
       <x:c r="D151" s="19"/>
       <x:c r="E151" s="19"/>
-      <x:c r="F151" s="16"/>
+      <x:c r="F151" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G151" s="22"/>
       <x:c r="H151" s="25"/>
     </x:row>
@@ -2057,7 +2357,9 @@
       <x:c r="C152" s="16"/>
       <x:c r="D152" s="19"/>
       <x:c r="E152" s="19"/>
-      <x:c r="F152" s="16"/>
+      <x:c r="F152" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G152" s="22"/>
       <x:c r="H152" s="25"/>
     </x:row>
@@ -2067,7 +2369,9 @@
       <x:c r="C153" s="16"/>
       <x:c r="D153" s="19"/>
       <x:c r="E153" s="19"/>
-      <x:c r="F153" s="16"/>
+      <x:c r="F153" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G153" s="22"/>
       <x:c r="H153" s="25"/>
     </x:row>
@@ -2077,7 +2381,9 @@
       <x:c r="C154" s="16"/>
       <x:c r="D154" s="19"/>
       <x:c r="E154" s="19"/>
-      <x:c r="F154" s="16"/>
+      <x:c r="F154" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G154" s="22"/>
       <x:c r="H154" s="25"/>
     </x:row>
@@ -2087,7 +2393,9 @@
       <x:c r="C155" s="16"/>
       <x:c r="D155" s="19"/>
       <x:c r="E155" s="19"/>
-      <x:c r="F155" s="16"/>
+      <x:c r="F155" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G155" s="22"/>
       <x:c r="H155" s="25"/>
     </x:row>
@@ -2097,7 +2405,9 @@
       <x:c r="C156" s="16"/>
       <x:c r="D156" s="19"/>
       <x:c r="E156" s="19"/>
-      <x:c r="F156" s="16"/>
+      <x:c r="F156" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G156" s="22"/>
       <x:c r="H156" s="25"/>
     </x:row>
@@ -2107,7 +2417,9 @@
       <x:c r="C157" s="16"/>
       <x:c r="D157" s="19"/>
       <x:c r="E157" s="19"/>
-      <x:c r="F157" s="16"/>
+      <x:c r="F157" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G157" s="22"/>
       <x:c r="H157" s="25"/>
     </x:row>
@@ -2117,7 +2429,9 @@
       <x:c r="C158" s="16"/>
       <x:c r="D158" s="19"/>
       <x:c r="E158" s="19"/>
-      <x:c r="F158" s="16"/>
+      <x:c r="F158" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G158" s="22"/>
       <x:c r="H158" s="25"/>
     </x:row>
@@ -2127,7 +2441,9 @@
       <x:c r="C159" s="16"/>
       <x:c r="D159" s="19"/>
       <x:c r="E159" s="19"/>
-      <x:c r="F159" s="16"/>
+      <x:c r="F159" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G159" s="22"/>
       <x:c r="H159" s="25"/>
     </x:row>
@@ -2137,7 +2453,9 @@
       <x:c r="C160" s="16"/>
       <x:c r="D160" s="19"/>
       <x:c r="E160" s="19"/>
-      <x:c r="F160" s="16"/>
+      <x:c r="F160" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G160" s="22"/>
       <x:c r="H160" s="25"/>
     </x:row>
@@ -2147,7 +2465,9 @@
       <x:c r="C161" s="16"/>
       <x:c r="D161" s="19"/>
       <x:c r="E161" s="19"/>
-      <x:c r="F161" s="16"/>
+      <x:c r="F161" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G161" s="22"/>
       <x:c r="H161" s="25"/>
     </x:row>
@@ -2157,7 +2477,9 @@
       <x:c r="C162" s="16"/>
       <x:c r="D162" s="19"/>
       <x:c r="E162" s="19"/>
-      <x:c r="F162" s="16"/>
+      <x:c r="F162" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G162" s="22"/>
       <x:c r="H162" s="25"/>
     </x:row>
@@ -2167,7 +2489,9 @@
       <x:c r="C163" s="16"/>
       <x:c r="D163" s="19"/>
       <x:c r="E163" s="19"/>
-      <x:c r="F163" s="16"/>
+      <x:c r="F163" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G163" s="22"/>
       <x:c r="H163" s="25"/>
     </x:row>
@@ -2177,7 +2501,9 @@
       <x:c r="C164" s="16"/>
       <x:c r="D164" s="19"/>
       <x:c r="E164" s="19"/>
-      <x:c r="F164" s="16"/>
+      <x:c r="F164" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G164" s="22"/>
       <x:c r="H164" s="25"/>
     </x:row>
@@ -2187,7 +2513,9 @@
       <x:c r="C165" s="16"/>
       <x:c r="D165" s="19"/>
       <x:c r="E165" s="19"/>
-      <x:c r="F165" s="16"/>
+      <x:c r="F165" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G165" s="22"/>
       <x:c r="H165" s="25"/>
     </x:row>
@@ -2197,7 +2525,9 @@
       <x:c r="C166" s="16"/>
       <x:c r="D166" s="19"/>
       <x:c r="E166" s="19"/>
-      <x:c r="F166" s="16"/>
+      <x:c r="F166" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G166" s="22"/>
       <x:c r="H166" s="25"/>
     </x:row>
@@ -2207,7 +2537,9 @@
       <x:c r="C167" s="16"/>
       <x:c r="D167" s="19"/>
       <x:c r="E167" s="19"/>
-      <x:c r="F167" s="16"/>
+      <x:c r="F167" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G167" s="22"/>
       <x:c r="H167" s="25"/>
     </x:row>
@@ -2217,7 +2549,9 @@
       <x:c r="C168" s="16"/>
       <x:c r="D168" s="19"/>
       <x:c r="E168" s="19"/>
-      <x:c r="F168" s="16"/>
+      <x:c r="F168" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G168" s="22"/>
       <x:c r="H168" s="25"/>
     </x:row>
@@ -2227,7 +2561,9 @@
       <x:c r="C169" s="16"/>
       <x:c r="D169" s="19"/>
       <x:c r="E169" s="19"/>
-      <x:c r="F169" s="16"/>
+      <x:c r="F169" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G169" s="22"/>
       <x:c r="H169" s="25"/>
     </x:row>
@@ -2237,7 +2573,9 @@
       <x:c r="C170" s="16"/>
       <x:c r="D170" s="19"/>
       <x:c r="E170" s="19"/>
-      <x:c r="F170" s="16"/>
+      <x:c r="F170" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G170" s="22"/>
       <x:c r="H170" s="25"/>
     </x:row>
@@ -2247,7 +2585,9 @@
       <x:c r="C171" s="16"/>
       <x:c r="D171" s="19"/>
       <x:c r="E171" s="19"/>
-      <x:c r="F171" s="16"/>
+      <x:c r="F171" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G171" s="22"/>
       <x:c r="H171" s="25"/>
     </x:row>
@@ -2257,7 +2597,9 @@
       <x:c r="C172" s="16"/>
       <x:c r="D172" s="19"/>
       <x:c r="E172" s="19"/>
-      <x:c r="F172" s="16"/>
+      <x:c r="F172" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G172" s="22"/>
       <x:c r="H172" s="25"/>
     </x:row>
@@ -2267,7 +2609,9 @@
       <x:c r="C173" s="16"/>
       <x:c r="D173" s="19"/>
       <x:c r="E173" s="19"/>
-      <x:c r="F173" s="16"/>
+      <x:c r="F173" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G173" s="22"/>
       <x:c r="H173" s="25"/>
     </x:row>
@@ -2277,7 +2621,9 @@
       <x:c r="C174" s="16"/>
       <x:c r="D174" s="19"/>
       <x:c r="E174" s="19"/>
-      <x:c r="F174" s="16"/>
+      <x:c r="F174" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G174" s="22"/>
       <x:c r="H174" s="25"/>
     </x:row>
@@ -2287,7 +2633,9 @@
       <x:c r="C175" s="16"/>
       <x:c r="D175" s="19"/>
       <x:c r="E175" s="19"/>
-      <x:c r="F175" s="16"/>
+      <x:c r="F175" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G175" s="22"/>
       <x:c r="H175" s="25"/>
     </x:row>
@@ -2297,7 +2645,9 @@
       <x:c r="C176" s="16"/>
       <x:c r="D176" s="19"/>
       <x:c r="E176" s="19"/>
-      <x:c r="F176" s="16"/>
+      <x:c r="F176" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G176" s="22"/>
       <x:c r="H176" s="25"/>
     </x:row>
@@ -2307,7 +2657,9 @@
       <x:c r="C177" s="16"/>
       <x:c r="D177" s="19"/>
       <x:c r="E177" s="19"/>
-      <x:c r="F177" s="16"/>
+      <x:c r="F177" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G177" s="22"/>
       <x:c r="H177" s="25"/>
     </x:row>
@@ -2317,7 +2669,9 @@
       <x:c r="C178" s="16"/>
       <x:c r="D178" s="19"/>
       <x:c r="E178" s="19"/>
-      <x:c r="F178" s="16"/>
+      <x:c r="F178" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G178" s="22"/>
       <x:c r="H178" s="25"/>
     </x:row>
@@ -2327,7 +2681,9 @@
       <x:c r="C179" s="16"/>
       <x:c r="D179" s="19"/>
       <x:c r="E179" s="19"/>
-      <x:c r="F179" s="16"/>
+      <x:c r="F179" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G179" s="22"/>
       <x:c r="H179" s="25"/>
     </x:row>
@@ -2337,7 +2693,9 @@
       <x:c r="C180" s="16"/>
       <x:c r="D180" s="19"/>
       <x:c r="E180" s="19"/>
-      <x:c r="F180" s="16"/>
+      <x:c r="F180" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G180" s="22"/>
       <x:c r="H180" s="25"/>
     </x:row>
@@ -2347,7 +2705,9 @@
       <x:c r="C181" s="16"/>
       <x:c r="D181" s="19"/>
       <x:c r="E181" s="19"/>
-      <x:c r="F181" s="16"/>
+      <x:c r="F181" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G181" s="22"/>
       <x:c r="H181" s="25"/>
     </x:row>
@@ -2357,7 +2717,9 @@
       <x:c r="C182" s="16"/>
       <x:c r="D182" s="19"/>
       <x:c r="E182" s="19"/>
-      <x:c r="F182" s="16"/>
+      <x:c r="F182" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G182" s="22"/>
       <x:c r="H182" s="25"/>
     </x:row>
@@ -2367,7 +2729,9 @@
       <x:c r="C183" s="16"/>
       <x:c r="D183" s="19"/>
       <x:c r="E183" s="19"/>
-      <x:c r="F183" s="16"/>
+      <x:c r="F183" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G183" s="22"/>
       <x:c r="H183" s="25"/>
     </x:row>
@@ -2377,7 +2741,9 @@
       <x:c r="C184" s="16"/>
       <x:c r="D184" s="19"/>
       <x:c r="E184" s="19"/>
-      <x:c r="F184" s="16"/>
+      <x:c r="F184" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G184" s="22"/>
       <x:c r="H184" s="25"/>
     </x:row>
@@ -2387,7 +2753,9 @@
       <x:c r="C185" s="16"/>
       <x:c r="D185" s="19"/>
       <x:c r="E185" s="19"/>
-      <x:c r="F185" s="16"/>
+      <x:c r="F185" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G185" s="22"/>
       <x:c r="H185" s="25"/>
     </x:row>
@@ -2397,7 +2765,9 @@
       <x:c r="C186" s="16"/>
       <x:c r="D186" s="19"/>
       <x:c r="E186" s="19"/>
-      <x:c r="F186" s="16"/>
+      <x:c r="F186" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G186" s="22"/>
       <x:c r="H186" s="25"/>
     </x:row>
@@ -2407,7 +2777,9 @@
       <x:c r="C187" s="16"/>
       <x:c r="D187" s="19"/>
       <x:c r="E187" s="19"/>
-      <x:c r="F187" s="16"/>
+      <x:c r="F187" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G187" s="22"/>
       <x:c r="H187" s="25"/>
     </x:row>
@@ -2417,7 +2789,9 @@
       <x:c r="C188" s="16"/>
       <x:c r="D188" s="19"/>
       <x:c r="E188" s="19"/>
-      <x:c r="F188" s="16"/>
+      <x:c r="F188" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G188" s="22"/>
       <x:c r="H188" s="25"/>
     </x:row>
@@ -2427,7 +2801,9 @@
       <x:c r="C189" s="16"/>
       <x:c r="D189" s="19"/>
       <x:c r="E189" s="19"/>
-      <x:c r="F189" s="16"/>
+      <x:c r="F189" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G189" s="22"/>
       <x:c r="H189" s="25"/>
     </x:row>
@@ -2437,7 +2813,9 @@
       <x:c r="C190" s="16"/>
       <x:c r="D190" s="19"/>
       <x:c r="E190" s="19"/>
-      <x:c r="F190" s="16"/>
+      <x:c r="F190" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G190" s="22"/>
       <x:c r="H190" s="25"/>
     </x:row>
@@ -2447,7 +2825,9 @@
       <x:c r="C191" s="16"/>
       <x:c r="D191" s="19"/>
       <x:c r="E191" s="19"/>
-      <x:c r="F191" s="16"/>
+      <x:c r="F191" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G191" s="22"/>
       <x:c r="H191" s="25"/>
     </x:row>
@@ -2457,7 +2837,9 @@
       <x:c r="C192" s="16"/>
       <x:c r="D192" s="19"/>
       <x:c r="E192" s="19"/>
-      <x:c r="F192" s="16"/>
+      <x:c r="F192" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G192" s="22"/>
       <x:c r="H192" s="25"/>
     </x:row>
@@ -2467,7 +2849,9 @@
       <x:c r="C193" s="16"/>
       <x:c r="D193" s="19"/>
       <x:c r="E193" s="19"/>
-      <x:c r="F193" s="16"/>
+      <x:c r="F193" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G193" s="22"/>
       <x:c r="H193" s="25"/>
     </x:row>
@@ -2477,7 +2861,9 @@
       <x:c r="C194" s="16"/>
       <x:c r="D194" s="19"/>
       <x:c r="E194" s="19"/>
-      <x:c r="F194" s="16"/>
+      <x:c r="F194" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G194" s="22"/>
       <x:c r="H194" s="25"/>
     </x:row>
@@ -2487,7 +2873,9 @@
       <x:c r="C195" s="16"/>
       <x:c r="D195" s="19"/>
       <x:c r="E195" s="19"/>
-      <x:c r="F195" s="16"/>
+      <x:c r="F195" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G195" s="22"/>
       <x:c r="H195" s="25"/>
     </x:row>
@@ -2497,7 +2885,9 @@
       <x:c r="C196" s="16"/>
       <x:c r="D196" s="19"/>
       <x:c r="E196" s="19"/>
-      <x:c r="F196" s="16"/>
+      <x:c r="F196" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G196" s="22"/>
       <x:c r="H196" s="25"/>
     </x:row>
@@ -2507,7 +2897,9 @@
       <x:c r="C197" s="16"/>
       <x:c r="D197" s="19"/>
       <x:c r="E197" s="19"/>
-      <x:c r="F197" s="16"/>
+      <x:c r="F197" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G197" s="22"/>
       <x:c r="H197" s="25"/>
     </x:row>
@@ -2517,7 +2909,9 @@
       <x:c r="C198" s="16"/>
       <x:c r="D198" s="19"/>
       <x:c r="E198" s="19"/>
-      <x:c r="F198" s="16"/>
+      <x:c r="F198" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G198" s="22"/>
       <x:c r="H198" s="25"/>
     </x:row>
@@ -2527,7 +2921,9 @@
       <x:c r="C199" s="16"/>
       <x:c r="D199" s="19"/>
       <x:c r="E199" s="19"/>
-      <x:c r="F199" s="16"/>
+      <x:c r="F199" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G199" s="22"/>
       <x:c r="H199" s="25"/>
     </x:row>
@@ -2537,7 +2933,9 @@
       <x:c r="C200" s="16"/>
       <x:c r="D200" s="19"/>
       <x:c r="E200" s="19"/>
-      <x:c r="F200" s="16"/>
+      <x:c r="F200" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G200" s="22"/>
       <x:c r="H200" s="25"/>
     </x:row>
@@ -2547,7 +2945,9 @@
       <x:c r="C201" s="16"/>
       <x:c r="D201" s="19"/>
       <x:c r="E201" s="19"/>
-      <x:c r="F201" s="16"/>
+      <x:c r="F201" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G201" s="22"/>
       <x:c r="H201" s="25"/>
     </x:row>
@@ -2557,7 +2957,9 @@
       <x:c r="C202" s="16"/>
       <x:c r="D202" s="19"/>
       <x:c r="E202" s="19"/>
-      <x:c r="F202" s="16"/>
+      <x:c r="F202" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G202" s="22"/>
       <x:c r="H202" s="25"/>
     </x:row>
@@ -2567,7 +2969,9 @@
       <x:c r="C203" s="16"/>
       <x:c r="D203" s="19"/>
       <x:c r="E203" s="19"/>
-      <x:c r="F203" s="16"/>
+      <x:c r="F203" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G203" s="22"/>
       <x:c r="H203" s="25"/>
     </x:row>
@@ -2577,7 +2981,9 @@
       <x:c r="C204" s="16"/>
       <x:c r="D204" s="19"/>
       <x:c r="E204" s="19"/>
-      <x:c r="F204" s="16"/>
+      <x:c r="F204" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G204" s="22"/>
       <x:c r="H204" s="25"/>
     </x:row>
@@ -2587,7 +2993,9 @@
       <x:c r="C205" s="16"/>
       <x:c r="D205" s="19"/>
       <x:c r="E205" s="19"/>
-      <x:c r="F205" s="16"/>
+      <x:c r="F205" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G205" s="22"/>
       <x:c r="H205" s="25"/>
     </x:row>
@@ -2597,7 +3005,9 @@
       <x:c r="C206" s="16"/>
       <x:c r="D206" s="19"/>
       <x:c r="E206" s="19"/>
-      <x:c r="F206" s="16"/>
+      <x:c r="F206" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G206" s="22"/>
       <x:c r="H206" s="25"/>
     </x:row>
@@ -2607,7 +3017,9 @@
       <x:c r="C207" s="16"/>
       <x:c r="D207" s="19"/>
       <x:c r="E207" s="19"/>
-      <x:c r="F207" s="16"/>
+      <x:c r="F207" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G207" s="22"/>
       <x:c r="H207" s="25"/>
     </x:row>
@@ -2617,7 +3029,9 @@
       <x:c r="C208" s="16"/>
       <x:c r="D208" s="19"/>
       <x:c r="E208" s="19"/>
-      <x:c r="F208" s="16"/>
+      <x:c r="F208" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G208" s="22"/>
       <x:c r="H208" s="25"/>
     </x:row>
@@ -2627,7 +3041,9 @@
       <x:c r="C209" s="16"/>
       <x:c r="D209" s="19"/>
       <x:c r="E209" s="19"/>
-      <x:c r="F209" s="16"/>
+      <x:c r="F209" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G209" s="22"/>
       <x:c r="H209" s="25"/>
     </x:row>
@@ -2637,7 +3053,9 @@
       <x:c r="C210" s="16"/>
       <x:c r="D210" s="19"/>
       <x:c r="E210" s="19"/>
-      <x:c r="F210" s="16"/>
+      <x:c r="F210" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G210" s="22"/>
       <x:c r="H210" s="25"/>
     </x:row>
@@ -2647,7 +3065,9 @@
       <x:c r="C211" s="16"/>
       <x:c r="D211" s="19"/>
       <x:c r="E211" s="19"/>
-      <x:c r="F211" s="16"/>
+      <x:c r="F211" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G211" s="22"/>
       <x:c r="H211" s="25"/>
     </x:row>
@@ -2657,7 +3077,9 @@
       <x:c r="C212" s="16"/>
       <x:c r="D212" s="19"/>
       <x:c r="E212" s="19"/>
-      <x:c r="F212" s="16"/>
+      <x:c r="F212" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G212" s="22"/>
       <x:c r="H212" s="25"/>
     </x:row>
@@ -2667,7 +3089,9 @@
       <x:c r="C213" s="16"/>
       <x:c r="D213" s="19"/>
       <x:c r="E213" s="19"/>
-      <x:c r="F213" s="16"/>
+      <x:c r="F213" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G213" s="22"/>
       <x:c r="H213" s="25"/>
     </x:row>
@@ -2677,7 +3101,9 @@
       <x:c r="C214" s="16"/>
       <x:c r="D214" s="19"/>
       <x:c r="E214" s="19"/>
-      <x:c r="F214" s="16"/>
+      <x:c r="F214" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G214" s="22"/>
       <x:c r="H214" s="25"/>
     </x:row>
@@ -2687,7 +3113,9 @@
       <x:c r="C215" s="16"/>
       <x:c r="D215" s="19"/>
       <x:c r="E215" s="19"/>
-      <x:c r="F215" s="16"/>
+      <x:c r="F215" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G215" s="22"/>
       <x:c r="H215" s="25"/>
     </x:row>
@@ -2697,7 +3125,9 @@
       <x:c r="C216" s="16"/>
       <x:c r="D216" s="19"/>
       <x:c r="E216" s="19"/>
-      <x:c r="F216" s="16"/>
+      <x:c r="F216" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G216" s="22"/>
       <x:c r="H216" s="25"/>
     </x:row>
@@ -2707,7 +3137,9 @@
       <x:c r="C217" s="16"/>
       <x:c r="D217" s="19"/>
       <x:c r="E217" s="19"/>
-      <x:c r="F217" s="16"/>
+      <x:c r="F217" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G217" s="22"/>
       <x:c r="H217" s="25"/>
     </x:row>
@@ -2717,7 +3149,9 @@
       <x:c r="C218" s="16"/>
       <x:c r="D218" s="19"/>
       <x:c r="E218" s="19"/>
-      <x:c r="F218" s="16"/>
+      <x:c r="F218" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G218" s="22"/>
       <x:c r="H218" s="25"/>
     </x:row>
@@ -2727,7 +3161,9 @@
       <x:c r="C219" s="16"/>
       <x:c r="D219" s="19"/>
       <x:c r="E219" s="19"/>
-      <x:c r="F219" s="16"/>
+      <x:c r="F219" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G219" s="22"/>
       <x:c r="H219" s="25"/>
     </x:row>
@@ -2737,7 +3173,9 @@
       <x:c r="C220" s="16"/>
       <x:c r="D220" s="19"/>
       <x:c r="E220" s="19"/>
-      <x:c r="F220" s="16"/>
+      <x:c r="F220" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G220" s="22"/>
       <x:c r="H220" s="25"/>
     </x:row>
@@ -2747,7 +3185,9 @@
       <x:c r="C221" s="16"/>
       <x:c r="D221" s="19"/>
       <x:c r="E221" s="19"/>
-      <x:c r="F221" s="16"/>
+      <x:c r="F221" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G221" s="22"/>
       <x:c r="H221" s="25"/>
     </x:row>
@@ -2757,7 +3197,9 @@
       <x:c r="C222" s="16"/>
       <x:c r="D222" s="19"/>
       <x:c r="E222" s="19"/>
-      <x:c r="F222" s="16"/>
+      <x:c r="F222" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G222" s="22"/>
       <x:c r="H222" s="25"/>
     </x:row>
@@ -2767,7 +3209,9 @@
       <x:c r="C223" s="16"/>
       <x:c r="D223" s="19"/>
       <x:c r="E223" s="19"/>
-      <x:c r="F223" s="16"/>
+      <x:c r="F223" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G223" s="22"/>
       <x:c r="H223" s="25"/>
     </x:row>
@@ -2777,7 +3221,9 @@
       <x:c r="C224" s="16"/>
       <x:c r="D224" s="19"/>
       <x:c r="E224" s="19"/>
-      <x:c r="F224" s="16"/>
+      <x:c r="F224" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G224" s="22"/>
       <x:c r="H224" s="25"/>
     </x:row>
@@ -2787,7 +3233,9 @@
       <x:c r="C225" s="16"/>
       <x:c r="D225" s="19"/>
       <x:c r="E225" s="19"/>
-      <x:c r="F225" s="16"/>
+      <x:c r="F225" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G225" s="22"/>
       <x:c r="H225" s="25"/>
     </x:row>
@@ -2797,7 +3245,9 @@
       <x:c r="C226" s="16"/>
       <x:c r="D226" s="19"/>
       <x:c r="E226" s="19"/>
-      <x:c r="F226" s="16"/>
+      <x:c r="F226" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G226" s="22"/>
       <x:c r="H226" s="25"/>
     </x:row>
@@ -2807,7 +3257,9 @@
       <x:c r="C227" s="16"/>
       <x:c r="D227" s="19"/>
       <x:c r="E227" s="19"/>
-      <x:c r="F227" s="16"/>
+      <x:c r="F227" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G227" s="22"/>
       <x:c r="H227" s="25"/>
     </x:row>
@@ -2817,7 +3269,9 @@
       <x:c r="C228" s="16"/>
       <x:c r="D228" s="19"/>
       <x:c r="E228" s="19"/>
-      <x:c r="F228" s="16"/>
+      <x:c r="F228" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G228" s="22"/>
       <x:c r="H228" s="25"/>
     </x:row>
@@ -2827,7 +3281,9 @@
       <x:c r="C229" s="16"/>
       <x:c r="D229" s="19"/>
       <x:c r="E229" s="19"/>
-      <x:c r="F229" s="16"/>
+      <x:c r="F229" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G229" s="22"/>
       <x:c r="H229" s="25"/>
     </x:row>
@@ -2837,7 +3293,9 @@
       <x:c r="C230" s="16"/>
       <x:c r="D230" s="19"/>
       <x:c r="E230" s="19"/>
-      <x:c r="F230" s="16"/>
+      <x:c r="F230" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G230" s="22"/>
       <x:c r="H230" s="25"/>
     </x:row>
@@ -2847,7 +3305,9 @@
       <x:c r="C231" s="16"/>
       <x:c r="D231" s="19"/>
       <x:c r="E231" s="19"/>
-      <x:c r="F231" s="16"/>
+      <x:c r="F231" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G231" s="22"/>
       <x:c r="H231" s="25"/>
     </x:row>
@@ -2857,7 +3317,9 @@
       <x:c r="C232" s="16"/>
       <x:c r="D232" s="19"/>
       <x:c r="E232" s="19"/>
-      <x:c r="F232" s="16"/>
+      <x:c r="F232" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G232" s="22"/>
       <x:c r="H232" s="25"/>
     </x:row>
@@ -2867,7 +3329,9 @@
       <x:c r="C233" s="16"/>
       <x:c r="D233" s="19"/>
       <x:c r="E233" s="19"/>
-      <x:c r="F233" s="16"/>
+      <x:c r="F233" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G233" s="22"/>
       <x:c r="H233" s="25"/>
     </x:row>
@@ -2877,7 +3341,9 @@
       <x:c r="C234" s="16"/>
       <x:c r="D234" s="19"/>
       <x:c r="E234" s="19"/>
-      <x:c r="F234" s="16"/>
+      <x:c r="F234" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G234" s="22"/>
       <x:c r="H234" s="25"/>
     </x:row>
@@ -2887,7 +3353,9 @@
       <x:c r="C235" s="16"/>
       <x:c r="D235" s="19"/>
       <x:c r="E235" s="19"/>
-      <x:c r="F235" s="16"/>
+      <x:c r="F235" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G235" s="22"/>
       <x:c r="H235" s="25"/>
     </x:row>
@@ -2897,7 +3365,9 @@
       <x:c r="C236" s="16"/>
       <x:c r="D236" s="19"/>
       <x:c r="E236" s="19"/>
-      <x:c r="F236" s="16"/>
+      <x:c r="F236" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G236" s="22"/>
       <x:c r="H236" s="25"/>
     </x:row>
@@ -2907,7 +3377,9 @@
       <x:c r="C237" s="16"/>
       <x:c r="D237" s="19"/>
       <x:c r="E237" s="19"/>
-      <x:c r="F237" s="16"/>
+      <x:c r="F237" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G237" s="22"/>
       <x:c r="H237" s="25"/>
     </x:row>
@@ -2917,7 +3389,9 @@
       <x:c r="C238" s="16"/>
       <x:c r="D238" s="19"/>
       <x:c r="E238" s="19"/>
-      <x:c r="F238" s="16"/>
+      <x:c r="F238" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G238" s="22"/>
       <x:c r="H238" s="25"/>
     </x:row>
@@ -2927,7 +3401,9 @@
       <x:c r="C239" s="16"/>
       <x:c r="D239" s="19"/>
       <x:c r="E239" s="19"/>
-      <x:c r="F239" s="16"/>
+      <x:c r="F239" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G239" s="22"/>
       <x:c r="H239" s="25"/>
     </x:row>
@@ -2937,7 +3413,9 @@
       <x:c r="C240" s="16"/>
       <x:c r="D240" s="19"/>
       <x:c r="E240" s="19"/>
-      <x:c r="F240" s="16"/>
+      <x:c r="F240" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G240" s="22"/>
       <x:c r="H240" s="25"/>
     </x:row>
@@ -2947,7 +3425,9 @@
       <x:c r="C241" s="16"/>
       <x:c r="D241" s="19"/>
       <x:c r="E241" s="19"/>
-      <x:c r="F241" s="16"/>
+      <x:c r="F241" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G241" s="22"/>
       <x:c r="H241" s="25"/>
     </x:row>
@@ -2957,7 +3437,9 @@
       <x:c r="C242" s="16"/>
       <x:c r="D242" s="19"/>
       <x:c r="E242" s="19"/>
-      <x:c r="F242" s="16"/>
+      <x:c r="F242" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G242" s="22"/>
       <x:c r="H242" s="25"/>
     </x:row>
@@ -2967,7 +3449,9 @@
       <x:c r="C243" s="16"/>
       <x:c r="D243" s="19"/>
       <x:c r="E243" s="19"/>
-      <x:c r="F243" s="16"/>
+      <x:c r="F243" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G243" s="22"/>
       <x:c r="H243" s="25"/>
     </x:row>
@@ -2977,7 +3461,9 @@
       <x:c r="C244" s="16"/>
       <x:c r="D244" s="19"/>
       <x:c r="E244" s="19"/>
-      <x:c r="F244" s="16"/>
+      <x:c r="F244" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G244" s="22"/>
       <x:c r="H244" s="25"/>
     </x:row>
@@ -2987,7 +3473,9 @@
       <x:c r="C245" s="16"/>
       <x:c r="D245" s="19"/>
       <x:c r="E245" s="19"/>
-      <x:c r="F245" s="16"/>
+      <x:c r="F245" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G245" s="22"/>
       <x:c r="H245" s="25"/>
     </x:row>
@@ -2997,7 +3485,9 @@
       <x:c r="C246" s="16"/>
       <x:c r="D246" s="19"/>
       <x:c r="E246" s="19"/>
-      <x:c r="F246" s="16"/>
+      <x:c r="F246" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G246" s="22"/>
       <x:c r="H246" s="25"/>
     </x:row>
@@ -3007,7 +3497,9 @@
       <x:c r="C247" s="16"/>
       <x:c r="D247" s="19"/>
       <x:c r="E247" s="19"/>
-      <x:c r="F247" s="16"/>
+      <x:c r="F247" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G247" s="22"/>
       <x:c r="H247" s="25"/>
     </x:row>
@@ -3017,7 +3509,9 @@
       <x:c r="C248" s="16"/>
       <x:c r="D248" s="19"/>
       <x:c r="E248" s="19"/>
-      <x:c r="F248" s="16"/>
+      <x:c r="F248" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G248" s="22"/>
       <x:c r="H248" s="25"/>
     </x:row>
@@ -3027,7 +3521,9 @@
       <x:c r="C249" s="16"/>
       <x:c r="D249" s="19"/>
       <x:c r="E249" s="19"/>
-      <x:c r="F249" s="16"/>
+      <x:c r="F249" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G249" s="22"/>
       <x:c r="H249" s="25"/>
     </x:row>
@@ -3037,7 +3533,9 @@
       <x:c r="C250" s="16"/>
       <x:c r="D250" s="19"/>
       <x:c r="E250" s="19"/>
-      <x:c r="F250" s="16"/>
+      <x:c r="F250" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G250" s="22"/>
       <x:c r="H250" s="25"/>
     </x:row>
@@ -3047,7 +3545,9 @@
       <x:c r="C251" s="16"/>
       <x:c r="D251" s="19"/>
       <x:c r="E251" s="19"/>
-      <x:c r="F251" s="16"/>
+      <x:c r="F251" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G251" s="22"/>
       <x:c r="H251" s="25"/>
     </x:row>
@@ -3057,7 +3557,9 @@
       <x:c r="C252" s="16"/>
       <x:c r="D252" s="19"/>
       <x:c r="E252" s="19"/>
-      <x:c r="F252" s="16"/>
+      <x:c r="F252" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G252" s="22"/>
       <x:c r="H252" s="25"/>
     </x:row>
@@ -3067,7 +3569,9 @@
       <x:c r="C253" s="16"/>
       <x:c r="D253" s="19"/>
       <x:c r="E253" s="19"/>
-      <x:c r="F253" s="16"/>
+      <x:c r="F253" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G253" s="22"/>
       <x:c r="H253" s="25"/>
     </x:row>
@@ -3077,7 +3581,9 @@
       <x:c r="C254" s="16"/>
       <x:c r="D254" s="19"/>
       <x:c r="E254" s="19"/>
-      <x:c r="F254" s="16"/>
+      <x:c r="F254" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G254" s="22"/>
       <x:c r="H254" s="25"/>
     </x:row>
@@ -3087,7 +3593,9 @@
       <x:c r="C255" s="16"/>
       <x:c r="D255" s="19"/>
       <x:c r="E255" s="19"/>
-      <x:c r="F255" s="16"/>
+      <x:c r="F255" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G255" s="22"/>
       <x:c r="H255" s="25"/>
     </x:row>
@@ -3097,7 +3605,9 @@
       <x:c r="C256" s="16"/>
       <x:c r="D256" s="19"/>
       <x:c r="E256" s="19"/>
-      <x:c r="F256" s="16"/>
+      <x:c r="F256" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G256" s="22"/>
       <x:c r="H256" s="25"/>
     </x:row>
@@ -3107,7 +3617,9 @@
       <x:c r="C257" s="16"/>
       <x:c r="D257" s="19"/>
       <x:c r="E257" s="19"/>
-      <x:c r="F257" s="16"/>
+      <x:c r="F257" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G257" s="22"/>
       <x:c r="H257" s="25"/>
     </x:row>
@@ -3117,7 +3629,9 @@
       <x:c r="C258" s="16"/>
       <x:c r="D258" s="19"/>
       <x:c r="E258" s="19"/>
-      <x:c r="F258" s="16"/>
+      <x:c r="F258" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G258" s="22"/>
       <x:c r="H258" s="25"/>
     </x:row>
@@ -3127,7 +3641,9 @@
       <x:c r="C259" s="16"/>
       <x:c r="D259" s="19"/>
       <x:c r="E259" s="19"/>
-      <x:c r="F259" s="16"/>
+      <x:c r="F259" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G259" s="22"/>
       <x:c r="H259" s="25"/>
     </x:row>
@@ -3137,7 +3653,9 @@
       <x:c r="C260" s="16"/>
       <x:c r="D260" s="19"/>
       <x:c r="E260" s="19"/>
-      <x:c r="F260" s="16"/>
+      <x:c r="F260" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G260" s="22"/>
       <x:c r="H260" s="25"/>
     </x:row>
@@ -3147,7 +3665,9 @@
       <x:c r="C261" s="16"/>
       <x:c r="D261" s="19"/>
       <x:c r="E261" s="19"/>
-      <x:c r="F261" s="16"/>
+      <x:c r="F261" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G261" s="22"/>
       <x:c r="H261" s="25"/>
     </x:row>
@@ -3157,7 +3677,9 @@
       <x:c r="C262" s="16"/>
       <x:c r="D262" s="19"/>
       <x:c r="E262" s="19"/>
-      <x:c r="F262" s="16"/>
+      <x:c r="F262" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G262" s="22"/>
       <x:c r="H262" s="25"/>
     </x:row>
@@ -3167,7 +3689,9 @@
       <x:c r="C263" s="16"/>
       <x:c r="D263" s="19"/>
       <x:c r="E263" s="19"/>
-      <x:c r="F263" s="16"/>
+      <x:c r="F263" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G263" s="22"/>
       <x:c r="H263" s="25"/>
     </x:row>
@@ -3177,7 +3701,9 @@
       <x:c r="C264" s="16"/>
       <x:c r="D264" s="19"/>
       <x:c r="E264" s="19"/>
-      <x:c r="F264" s="16"/>
+      <x:c r="F264" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G264" s="22"/>
       <x:c r="H264" s="25"/>
     </x:row>
@@ -3187,7 +3713,9 @@
       <x:c r="C265" s="16"/>
       <x:c r="D265" s="19"/>
       <x:c r="E265" s="19"/>
-      <x:c r="F265" s="16"/>
+      <x:c r="F265" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G265" s="22"/>
       <x:c r="H265" s="25"/>
     </x:row>
@@ -3197,7 +3725,9 @@
       <x:c r="C266" s="16"/>
       <x:c r="D266" s="19"/>
       <x:c r="E266" s="19"/>
-      <x:c r="F266" s="16"/>
+      <x:c r="F266" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G266" s="22"/>
       <x:c r="H266" s="25"/>
     </x:row>
@@ -3207,7 +3737,9 @@
       <x:c r="C267" s="16"/>
       <x:c r="D267" s="19"/>
       <x:c r="E267" s="19"/>
-      <x:c r="F267" s="16"/>
+      <x:c r="F267" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G267" s="22"/>
       <x:c r="H267" s="25"/>
     </x:row>
@@ -3217,7 +3749,9 @@
       <x:c r="C268" s="16"/>
       <x:c r="D268" s="19"/>
       <x:c r="E268" s="19"/>
-      <x:c r="F268" s="16"/>
+      <x:c r="F268" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G268" s="22"/>
       <x:c r="H268" s="25"/>
     </x:row>
@@ -3227,7 +3761,9 @@
       <x:c r="C269" s="16"/>
       <x:c r="D269" s="19"/>
       <x:c r="E269" s="19"/>
-      <x:c r="F269" s="16"/>
+      <x:c r="F269" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G269" s="22"/>
       <x:c r="H269" s="25"/>
     </x:row>
@@ -3237,7 +3773,9 @@
       <x:c r="C270" s="16"/>
       <x:c r="D270" s="19"/>
       <x:c r="E270" s="19"/>
-      <x:c r="F270" s="16"/>
+      <x:c r="F270" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G270" s="22"/>
       <x:c r="H270" s="25"/>
     </x:row>
@@ -3247,7 +3785,9 @@
       <x:c r="C271" s="16"/>
       <x:c r="D271" s="19"/>
       <x:c r="E271" s="19"/>
-      <x:c r="F271" s="16"/>
+      <x:c r="F271" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G271" s="22"/>
       <x:c r="H271" s="25"/>
     </x:row>
@@ -3257,7 +3797,9 @@
       <x:c r="C272" s="16"/>
       <x:c r="D272" s="19"/>
       <x:c r="E272" s="19"/>
-      <x:c r="F272" s="16"/>
+      <x:c r="F272" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G272" s="22"/>
       <x:c r="H272" s="25"/>
     </x:row>
@@ -3267,7 +3809,9 @@
       <x:c r="C273" s="16"/>
       <x:c r="D273" s="19"/>
       <x:c r="E273" s="19"/>
-      <x:c r="F273" s="16"/>
+      <x:c r="F273" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G273" s="22"/>
       <x:c r="H273" s="25"/>
     </x:row>
@@ -3277,7 +3821,9 @@
       <x:c r="C274" s="16"/>
       <x:c r="D274" s="19"/>
       <x:c r="E274" s="19"/>
-      <x:c r="F274" s="16"/>
+      <x:c r="F274" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G274" s="22"/>
       <x:c r="H274" s="25"/>
     </x:row>
@@ -3287,7 +3833,9 @@
       <x:c r="C275" s="16"/>
       <x:c r="D275" s="19"/>
       <x:c r="E275" s="19"/>
-      <x:c r="F275" s="16"/>
+      <x:c r="F275" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G275" s="22"/>
       <x:c r="H275" s="25"/>
     </x:row>
@@ -3297,7 +3845,9 @@
       <x:c r="C276" s="16"/>
       <x:c r="D276" s="19"/>
       <x:c r="E276" s="19"/>
-      <x:c r="F276" s="16"/>
+      <x:c r="F276" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G276" s="22"/>
       <x:c r="H276" s="25"/>
     </x:row>
@@ -3307,7 +3857,9 @@
       <x:c r="C277" s="16"/>
       <x:c r="D277" s="19"/>
       <x:c r="E277" s="19"/>
-      <x:c r="F277" s="16"/>
+      <x:c r="F277" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G277" s="22"/>
       <x:c r="H277" s="25"/>
     </x:row>
@@ -3317,7 +3869,9 @@
       <x:c r="C278" s="16"/>
       <x:c r="D278" s="19"/>
       <x:c r="E278" s="19"/>
-      <x:c r="F278" s="16"/>
+      <x:c r="F278" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G278" s="22"/>
       <x:c r="H278" s="25"/>
     </x:row>
@@ -3327,7 +3881,9 @@
       <x:c r="C279" s="16"/>
       <x:c r="D279" s="19"/>
       <x:c r="E279" s="19"/>
-      <x:c r="F279" s="16"/>
+      <x:c r="F279" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G279" s="22"/>
       <x:c r="H279" s="25"/>
     </x:row>
@@ -3337,7 +3893,9 @@
       <x:c r="C280" s="16"/>
       <x:c r="D280" s="19"/>
       <x:c r="E280" s="19"/>
-      <x:c r="F280" s="16"/>
+      <x:c r="F280" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G280" s="22"/>
       <x:c r="H280" s="25"/>
     </x:row>
@@ -3347,7 +3905,9 @@
       <x:c r="C281" s="16"/>
       <x:c r="D281" s="19"/>
       <x:c r="E281" s="19"/>
-      <x:c r="F281" s="16"/>
+      <x:c r="F281" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G281" s="22"/>
       <x:c r="H281" s="25"/>
     </x:row>
@@ -3357,7 +3917,9 @@
       <x:c r="C282" s="16"/>
       <x:c r="D282" s="19"/>
       <x:c r="E282" s="19"/>
-      <x:c r="F282" s="16"/>
+      <x:c r="F282" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G282" s="22"/>
       <x:c r="H282" s="25"/>
     </x:row>
@@ -3367,7 +3929,9 @@
       <x:c r="C283" s="16"/>
       <x:c r="D283" s="19"/>
       <x:c r="E283" s="19"/>
-      <x:c r="F283" s="16"/>
+      <x:c r="F283" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G283" s="22"/>
       <x:c r="H283" s="25"/>
     </x:row>
@@ -3377,7 +3941,9 @@
       <x:c r="C284" s="16"/>
       <x:c r="D284" s="19"/>
       <x:c r="E284" s="19"/>
-      <x:c r="F284" s="16"/>
+      <x:c r="F284" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G284" s="22"/>
       <x:c r="H284" s="25"/>
     </x:row>
@@ -3387,7 +3953,9 @@
       <x:c r="C285" s="16"/>
       <x:c r="D285" s="19"/>
       <x:c r="E285" s="19"/>
-      <x:c r="F285" s="16"/>
+      <x:c r="F285" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G285" s="22"/>
       <x:c r="H285" s="25"/>
     </x:row>
@@ -3397,7 +3965,9 @@
       <x:c r="C286" s="16"/>
       <x:c r="D286" s="19"/>
       <x:c r="E286" s="19"/>
-      <x:c r="F286" s="16"/>
+      <x:c r="F286" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G286" s="22"/>
       <x:c r="H286" s="25"/>
     </x:row>
@@ -3407,7 +3977,9 @@
       <x:c r="C287" s="16"/>
       <x:c r="D287" s="19"/>
       <x:c r="E287" s="19"/>
-      <x:c r="F287" s="16"/>
+      <x:c r="F287" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G287" s="22"/>
       <x:c r="H287" s="25"/>
     </x:row>
@@ -3417,7 +3989,9 @@
       <x:c r="C288" s="16"/>
       <x:c r="D288" s="19"/>
       <x:c r="E288" s="19"/>
-      <x:c r="F288" s="16"/>
+      <x:c r="F288" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G288" s="22"/>
       <x:c r="H288" s="25"/>
     </x:row>
@@ -3427,7 +4001,9 @@
       <x:c r="C289" s="16"/>
       <x:c r="D289" s="19"/>
       <x:c r="E289" s="19"/>
-      <x:c r="F289" s="16"/>
+      <x:c r="F289" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G289" s="22"/>
       <x:c r="H289" s="25"/>
     </x:row>
@@ -3437,7 +4013,9 @@
       <x:c r="C290" s="16"/>
       <x:c r="D290" s="19"/>
       <x:c r="E290" s="19"/>
-      <x:c r="F290" s="16"/>
+      <x:c r="F290" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G290" s="22"/>
       <x:c r="H290" s="25"/>
     </x:row>
@@ -3447,7 +4025,9 @@
       <x:c r="C291" s="16"/>
       <x:c r="D291" s="19"/>
       <x:c r="E291" s="19"/>
-      <x:c r="F291" s="16"/>
+      <x:c r="F291" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G291" s="22"/>
       <x:c r="H291" s="25"/>
     </x:row>
@@ -3457,7 +4037,9 @@
       <x:c r="C292" s="16"/>
       <x:c r="D292" s="19"/>
       <x:c r="E292" s="19"/>
-      <x:c r="F292" s="16"/>
+      <x:c r="F292" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G292" s="22"/>
       <x:c r="H292" s="25"/>
     </x:row>
@@ -3467,7 +4049,9 @@
       <x:c r="C293" s="16"/>
       <x:c r="D293" s="19"/>
       <x:c r="E293" s="19"/>
-      <x:c r="F293" s="16"/>
+      <x:c r="F293" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G293" s="22"/>
       <x:c r="H293" s="25"/>
     </x:row>
@@ -3477,7 +4061,9 @@
       <x:c r="C294" s="16"/>
       <x:c r="D294" s="19"/>
       <x:c r="E294" s="19"/>
-      <x:c r="F294" s="16"/>
+      <x:c r="F294" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G294" s="22"/>
       <x:c r="H294" s="25"/>
     </x:row>
@@ -3487,7 +4073,9 @@
       <x:c r="C295" s="16"/>
       <x:c r="D295" s="19"/>
       <x:c r="E295" s="19"/>
-      <x:c r="F295" s="16"/>
+      <x:c r="F295" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G295" s="22"/>
       <x:c r="H295" s="25"/>
     </x:row>
@@ -3497,7 +4085,9 @@
       <x:c r="C296" s="16"/>
       <x:c r="D296" s="19"/>
       <x:c r="E296" s="19"/>
-      <x:c r="F296" s="16"/>
+      <x:c r="F296" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G296" s="22"/>
       <x:c r="H296" s="25"/>
     </x:row>
@@ -3507,7 +4097,9 @@
       <x:c r="C297" s="16"/>
       <x:c r="D297" s="19"/>
       <x:c r="E297" s="19"/>
-      <x:c r="F297" s="16"/>
+      <x:c r="F297" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G297" s="22"/>
       <x:c r="H297" s="25"/>
     </x:row>
@@ -3517,7 +4109,9 @@
       <x:c r="C298" s="16"/>
       <x:c r="D298" s="19"/>
       <x:c r="E298" s="19"/>
-      <x:c r="F298" s="16"/>
+      <x:c r="F298" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G298" s="22"/>
       <x:c r="H298" s="25"/>
     </x:row>
@@ -3527,7 +4121,9 @@
       <x:c r="C299" s="16"/>
       <x:c r="D299" s="19"/>
       <x:c r="E299" s="19"/>
-      <x:c r="F299" s="16"/>
+      <x:c r="F299" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G299" s="22"/>
       <x:c r="H299" s="25"/>
     </x:row>
@@ -3537,7 +4133,9 @@
       <x:c r="C300" s="16"/>
       <x:c r="D300" s="19"/>
       <x:c r="E300" s="19"/>
-      <x:c r="F300" s="16"/>
+      <x:c r="F300" s="16" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G300" s="22"/>
       <x:c r="H300" s="25"/>
     </x:row>
@@ -3547,7 +4145,9 @@
       <x:c r="C301" s="17"/>
       <x:c r="D301" s="20"/>
       <x:c r="E301" s="20"/>
-      <x:c r="F301" s="17"/>
+      <x:c r="F301" s="17" t="str">
+        <x:v>480×380×350</x:v>
+      </x:c>
       <x:c r="G301" s="23"/>
       <x:c r="H301" s="26"/>
     </x:row>
@@ -3581,7 +4181,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="28" t="str">
-        <x:v>浙江美集实业有限公司 · 集装箱装柜规划 · Excel 导入模板 v2.4</x:v>
+        <x:v>浙江美集实业有限公司 · 集装箱装柜规划 · Excel 导入模板 v2.5</x:v>
       </x:c>
       <x:c r="B1" s="28"/>
       <x:c r="C1" s="28"/>
@@ -3648,7 +4248,7 @@
         <x:v>外箱尺寸</x:v>
       </x:c>
       <x:c r="B11" s="45" t="str">
-        <x:v>必填；按 L×W×H 填写，例如 480×380×350，单位 mm；H 始终向上。</x:v>
+        <x:v>美集默认 480×380×350 mm，模板已预填；如有实测专用尺寸可覆盖。H 始终向上。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="29" customHeight="1">
@@ -3719,7 +4319,7 @@
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="56" t="str">
-        <x:v>数据仅在当前浏览器本地解析和保存。导入前请确认纸箱高度向上、尺寸为实测外廓；托盘包装请填写平底托盘实际尺寸。</x:v>
+        <x:v>数据仅在当前浏览器本地解析和保存。美集外箱缺省为 480×380×350 mm；若 SKU 有明确实测尺寸则以实测值覆盖。托盘包装请填写平底托盘实际尺寸。</x:v>
       </x:c>
       <x:c r="B20" s="56"/>
       <x:c r="C20" s="56"/>

</xml_diff>